<commit_message>
Make dialog box user settings persistent by adding a settings sheet to remember selections
</commit_message>
<xml_diff>
--- a/Right Triangles Example.xlsx
+++ b/Right Triangles Example.xlsx
@@ -8,13 +8,23 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\OneDrive - DataSoar\Projects\Excel_Steps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD322F2E-4648-44D2-B8D5-1CC1691606A0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0DFE4A6-480D-4697-B6D1-6179A1838654}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23212" yWindow="4133" windowWidth="10192" windowHeight="7687" xr2:uid="{5BB9F994-731B-4549-BC83-1B8B5E1EEF0D}"/>
+    <workbookView xWindow="-32543" yWindow="1238" windowWidth="26775" windowHeight="14865" activeTab="2" xr2:uid="{5BB9F994-731B-4549-BC83-1B8B5E1EEF0D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Triangles" sheetId="27" r:id="rId1"/>
+    <sheet name="Triangles" sheetId="34" r:id="rId1"/>
+    <sheet name="Example Steps" sheetId="28" r:id="rId2"/>
+    <sheet name="XLStepsSettings" sheetId="32" r:id="rId3"/>
+    <sheet name="ExcelSteps" sheetId="33" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName name="Description">Triangles!$A:$A</definedName>
+    <definedName name="Side_a">Triangles!$B:$B</definedName>
+    <definedName name="Side_b">Triangles!$C:$C</definedName>
+    <definedName name="Triangles">Triangles!$A:$C</definedName>
+    <definedName name="Triangles_Header">Triangles!$1:$1</definedName>
+  </definedNames>
   <calcPr calcId="191029" calcMode="manual"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -31,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
   <si>
     <t>Description</t>
   </si>
@@ -49,13 +59,67 @@
   </si>
   <si>
     <t>Side_b</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>txtval</t>
+  </si>
+  <si>
+    <t>boolean1</t>
+  </si>
+  <si>
+    <t>Sheet</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>Step</t>
+  </si>
+  <si>
+    <t>Formula/List Name/Sort-by</t>
+  </si>
+  <si>
+    <t>After or End Column</t>
+  </si>
+  <si>
+    <t>Keep Formulas</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Number Format</t>
+  </si>
+  <si>
+    <t>Width</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>boolean2</t>
+  </si>
+  <si>
+    <t>ShtNameFrm</t>
+  </si>
+  <si>
+    <t>Triangles</t>
+  </si>
+  <si>
+    <t>cBoxAppShtName</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -63,16 +127,47 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -80,15 +175,60 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="2" tint="-0.249977111117893"/>
+      </left>
+      <right style="thin">
+        <color theme="2" tint="-0.249977111117893"/>
+      </right>
+      <top style="thin">
+        <color theme="2" tint="-0.249977111117893"/>
+      </top>
+      <bottom style="thin">
+        <color theme="2" tint="-0.249977111117893"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Accent1" xfId="1" builtinId="29"/>
+    <cellStyle name="Accent2" xfId="2" builtinId="33"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -102,6 +242,61 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>167330</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C1DA1DA6-F1A9-45BF-9182-1620B36CF7FF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="647700" y="361950"/>
+          <a:ext cx="10058400" cy="1977080"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -400,64 +595,306 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C810996-6E3E-474B-B499-FAB0F4F68954}">
-  <sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B10E36F-1AF7-4DD5-9D70-FA4FA289E891}">
+  <sheetPr codeName="Sheet8">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="7.86328125" customWidth="1"/>
-    <col min="3" max="3" width="7.9296875" customWidth="1"/>
-    <col min="7" max="16384" width="9.06640625" style="1"/>
+    <col min="1" max="1" width="12" style="1" customWidth="1"/>
+    <col min="2" max="2" width="7.86328125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="7.9296875" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="9.06640625" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="13" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+      <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="12">
         <v>3</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="12">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+      <c r="A3" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="12">
         <v>6</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="12">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
+      <c r="A4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="12">
         <v>25</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="12">
         <v>50</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD0F7AA2-842E-45B4-A167-06F6B4024001}">
+  <sheetPr codeName="Sheet2"/>
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41325C8C-C6D7-402D-9E03-A497557690D4}">
+  <sheetPr codeName="Sheet6"/>
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="2" width="14.86328125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" t="b">
+        <v>1</v>
+      </c>
+      <c r="E2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C5D1086-8A1D-4E9F-A43C-00623B057C9E}">
+  <sheetPr codeName="Sheet7"/>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="3" width="12.59765625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="20.59765625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="12.59765625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="7.59765625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="12.59765625" style="11" customWidth="1"/>
+    <col min="8" max="8" width="7.59765625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="7.59765625" style="4" customWidth="1"/>
+    <col min="10" max="16384" width="9.06640625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="24" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="6"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="6"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="6"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="6"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C10" xr:uid="{22CFD59B-AF0E-4FD2-A694-25304071EC94}">
+      <formula1>"Col_Format, Col_Insert, Col_AddGroup, Col_Comment,Col_CondFormat, Col_Dropdown, Col_NumFormat, Col_Width, Tbl_FreezeRow1, Tbl_Sort"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Bug fix to FreezeRow1 command; update for Pandas compatibility; update Triangles case study based on MS Excel Jan 2020 update
</commit_message>
<xml_diff>
--- a/Right Triangles Example.xlsx
+++ b/Right Triangles Example.xlsx
@@ -1,31 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\OneDrive - DataSoar\Projects\Excel_Steps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0DFE4A6-480D-4697-B6D1-6179A1838654}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA6AE964-0C33-4855-9CBA-3803233E8726}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-32543" yWindow="1238" windowWidth="26775" windowHeight="14865" activeTab="2" xr2:uid="{5BB9F994-731B-4549-BC83-1B8B5E1EEF0D}"/>
+    <workbookView xWindow="1388" yWindow="1388" windowWidth="10485" windowHeight="8549" xr2:uid="{5BB9F994-731B-4549-BC83-1B8B5E1EEF0D}"/>
   </bookViews>
   <sheets>
-    <sheet name="Triangles" sheetId="34" r:id="rId1"/>
-    <sheet name="Example Steps" sheetId="28" r:id="rId2"/>
-    <sheet name="XLStepsSettings" sheetId="32" r:id="rId3"/>
-    <sheet name="ExcelSteps" sheetId="33" r:id="rId4"/>
+    <sheet name="Triangles" sheetId="39" r:id="rId1"/>
+    <sheet name="ExcelSteps" sheetId="33" r:id="rId2"/>
+    <sheet name="Example Steps" sheetId="28" r:id="rId3"/>
+    <sheet name="XLStepsSettings" sheetId="37" state="veryHidden" r:id="rId4"/>
   </sheets>
-  <definedNames>
-    <definedName name="Description">Triangles!$A:$A</definedName>
-    <definedName name="Side_a">Triangles!$B:$B</definedName>
-    <definedName name="Side_b">Triangles!$C:$C</definedName>
-    <definedName name="Triangles">Triangles!$A:$C</definedName>
-    <definedName name="Triangles_Header">Triangles!$1:$1</definedName>
-  </definedNames>
-  <calcPr calcId="191029" calcMode="manual"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -33,7 +26,9 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -41,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
   <si>
     <t>Description</t>
   </si>
@@ -61,7 +56,37 @@
     <t>Side_b</t>
   </si>
   <si>
-    <t>Name</t>
+    <t>Sheet</t>
+  </si>
+  <si>
+    <t>Column</t>
+  </si>
+  <si>
+    <t>Step</t>
+  </si>
+  <si>
+    <t>Formula/List Name/Sort-by</t>
+  </si>
+  <si>
+    <t>After or End Column</t>
+  </si>
+  <si>
+    <t>Keep Formulas</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Number Format</t>
+  </si>
+  <si>
+    <t>Width</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Triangles</t>
   </si>
   <si>
     <t>Type</t>
@@ -73,43 +98,13 @@
     <t>boolean1</t>
   </si>
   <si>
-    <t>Sheet</t>
-  </si>
-  <si>
-    <t>Column</t>
-  </si>
-  <si>
-    <t>Step</t>
-  </si>
-  <si>
-    <t>Formula/List Name/Sort-by</t>
-  </si>
-  <si>
-    <t>After or End Column</t>
-  </si>
-  <si>
-    <t>Keep Formulas</t>
-  </si>
-  <si>
-    <t>Comment</t>
-  </si>
-  <si>
-    <t>Number Format</t>
-  </si>
-  <si>
-    <t>Width</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>boolean2</t>
   </si>
   <si>
     <t>ShtNameFrm</t>
   </si>
   <si>
-    <t>Triangles</t>
+    <t>Example Steps</t>
   </si>
   <si>
     <t>cBoxAppShtName</t>
@@ -149,17 +144,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -191,18 +181,17 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
@@ -221,14 +210,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Accent1" xfId="1" builtinId="29"/>
-    <cellStyle name="Accent2" xfId="2" builtinId="33"/>
+  <cellStyles count="2">
+    <cellStyle name="Accent2" xfId="1" builtinId="33"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -250,21 +234,21 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
+      <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
       <xdr:colOff>342900</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>167330</xdr:rowOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>49429</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2">
+        <xdr:cNvPr id="4" name="Picture 3">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C1DA1DA6-F1A9-45BF-9182-1620B36CF7FF}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{14700AB2-DF6E-48C8-8F19-E0102C571C51}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -286,8 +270,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="647700" y="361950"/>
-          <a:ext cx="10058400" cy="1977080"/>
+          <a:off x="647700" y="180975"/>
+          <a:ext cx="10058400" cy="1678204"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -595,60 +579,59 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B10E36F-1AF7-4DD5-9D70-FA4FA289E891}">
-  <sheetPr codeName="Sheet8">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{579BDF3B-B142-41F6-B0EF-B33FE704109C}">
+  <sheetPr codeName="Sheet5">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="12" style="1" customWidth="1"/>
-    <col min="2" max="2" width="7.86328125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="7.9296875" style="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.06640625" style="1"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="7.86328125" customWidth="1"/>
+    <col min="3" max="3" width="7.9296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A1" s="13" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13" t="s">
+      <c r="B1" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="13" t="s">
+      <c r="C1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A2" s="12" t="s">
+      <c r="A2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="12">
+      <c r="B2">
         <v>3</v>
       </c>
-      <c r="C2" s="12">
+      <c r="C2">
         <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A3" s="12" t="s">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="12">
+      <c r="B3">
         <v>6</v>
       </c>
-      <c r="C3" s="12">
+      <c r="C3">
         <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A4" s="12" t="s">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="12">
+      <c r="B4">
         <v>25</v>
       </c>
-      <c r="C4" s="12">
+      <c r="C4">
         <v>50</v>
       </c>
     </row>
@@ -658,6 +641,166 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C5D1086-8A1D-4E9F-A43C-00623B057C9E}">
+  <sheetPr codeName="Sheet7"/>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="3" width="12.59765625" style="4" customWidth="1"/>
+    <col min="4" max="4" width="22.9296875" style="9" customWidth="1"/>
+    <col min="5" max="5" width="12.59765625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="7.59765625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="20.59765625" style="11" customWidth="1"/>
+    <col min="8" max="8" width="7.59765625" style="5" customWidth="1"/>
+    <col min="9" max="9" width="7.59765625" style="4" customWidth="1"/>
+    <col min="10" max="16384" width="9.06640625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="24" x14ac:dyDescent="0.45">
+      <c r="A1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A2" s="6"/>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="6"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="6"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A4" s="6"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="10"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A5" s="6"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="6"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A7" s="6"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="6"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C9" xr:uid="{22CFD59B-AF0E-4FD2-A694-25304071EC94}">
+      <formula1>"Col_Format, Col_Insert, Col_AddGroup, Col_Comment,Col_CondFormat, Col_Dropdown, Col_NumFormat, Col_Width, Tbl_FreezeRow1, Tbl_Sort"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="0" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD0F7AA2-842E-45B4-A167-06F6B4024001}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1"/>
@@ -668,233 +811,63 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41325C8C-C6D7-402D-9E03-A497557690D4}">
-  <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:E3"/>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF060701-7CA0-45C0-BD16-F41A6A5DB4E0}">
+  <sheetPr codeName="Sheet1"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="1" max="2" width="14.86328125" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="C1" t="s">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="D1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>21</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" t="s">
-        <v>22</v>
+        <v>16</v>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
       </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>23</v>
       </c>
-      <c r="B3" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" t="b">
-        <v>1</v>
+      <c r="C3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" t="b">
+        <v>0</v>
+      </c>
+      <c r="D4" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C5D1086-8A1D-4E9F-A43C-00623B057C9E}">
-  <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:I10"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="1" max="3" width="12.59765625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="20.59765625" style="9" customWidth="1"/>
-    <col min="5" max="5" width="12.59765625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="7.59765625" style="4" customWidth="1"/>
-    <col min="7" max="7" width="12.59765625" style="11" customWidth="1"/>
-    <col min="8" max="8" width="7.59765625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="7.59765625" style="4" customWidth="1"/>
-    <col min="10" max="16384" width="9.06640625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" ht="24" x14ac:dyDescent="0.45">
-      <c r="A1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="6"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="6"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="6"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="6"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="6"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="6"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="6"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="6"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="6"/>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C10" xr:uid="{22CFD59B-AF0E-4FD2-A694-25304071EC94}">
-      <formula1>"Col_Format, Col_Insert, Col_AddGroup, Col_Comment,Col_CondFormat, Col_Dropdown, Col_NumFormat, Col_Width, Tbl_FreezeRow1, Tbl_Sort"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Minor bug fix to format wide columns without crash; added Vimeo link to Readme
</commit_message>
<xml_diff>
--- a/Right Triangles Example.xlsx
+++ b/Right Triangles Example.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\Mac\Home\OneDrive - DataSoar\Projects\Excel_Steps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA6AE964-0C33-4855-9CBA-3803233E8726}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE6E809-C6BC-4D47-B8E3-52E1DCCE8C3E}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1388" yWindow="1388" windowWidth="10485" windowHeight="8549" xr2:uid="{5BB9F994-731B-4549-BC83-1B8B5E1EEF0D}"/>
+    <workbookView xWindow="1567" yWindow="1418" windowWidth="25313" windowHeight="15382" xr2:uid="{5BB9F994-731B-4549-BC83-1B8B5E1EEF0D}"/>
   </bookViews>
   <sheets>
     <sheet name="Triangles" sheetId="39" r:id="rId1"/>
-    <sheet name="ExcelSteps" sheetId="33" r:id="rId2"/>
-    <sheet name="Example Steps" sheetId="28" r:id="rId3"/>
-    <sheet name="XLStepsSettings" sheetId="37" state="veryHidden" r:id="rId4"/>
+    <sheet name="Example Steps" sheetId="28" r:id="rId2"/>
+    <sheet name="XLStepsSettings" sheetId="37" state="veryHidden" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="14">
   <si>
     <t>Description</t>
   </si>
@@ -54,36 +53,6 @@
   </si>
   <si>
     <t>Side_b</t>
-  </si>
-  <si>
-    <t>Sheet</t>
-  </si>
-  <si>
-    <t>Column</t>
-  </si>
-  <si>
-    <t>Step</t>
-  </si>
-  <si>
-    <t>Formula/List Name/Sort-by</t>
-  </si>
-  <si>
-    <t>After or End Column</t>
-  </si>
-  <si>
-    <t>Keep Formulas</t>
-  </si>
-  <si>
-    <t>Comment</t>
-  </si>
-  <si>
-    <t>Number Format</t>
-  </si>
-  <si>
-    <t>Width</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Triangles</t>
@@ -114,7 +83,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,42 +91,16 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -165,54 +108,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </left>
-      <right style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </right>
-      <top style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </top>
-      <bottom style="thin">
-        <color theme="2" tint="-0.249977111117893"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Accent2" xfId="1" builtinId="33"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -641,166 +544,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C5D1086-8A1D-4E9F-A43C-00623B057C9E}">
-  <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <cols>
-    <col min="1" max="3" width="12.59765625" style="4" customWidth="1"/>
-    <col min="4" max="4" width="22.9296875" style="9" customWidth="1"/>
-    <col min="5" max="5" width="12.59765625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="7.59765625" style="4" customWidth="1"/>
-    <col min="7" max="7" width="20.59765625" style="11" customWidth="1"/>
-    <col min="8" max="8" width="7.59765625" style="5" customWidth="1"/>
-    <col min="9" max="9" width="7.59765625" style="4" customWidth="1"/>
-    <col min="10" max="16384" width="9.06640625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:9" ht="24" x14ac:dyDescent="0.45">
-      <c r="A1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I1" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="6"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="6"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="6"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="6"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" s="6"/>
-      <c r="F6" s="6"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="6"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="6"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="6"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="6"/>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C9" xr:uid="{22CFD59B-AF0E-4FD2-A694-25304071EC94}">
-      <formula1>"Col_Format, Col_Insert, Col_AddGroup, Col_Comment,Col_CondFormat, Col_Dropdown, Col_NumFormat, Col_Width, Tbl_FreezeRow1, Tbl_Sort"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="0" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD0F7AA2-842E-45B4-A167-06F6B4024001}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1"/>
@@ -811,7 +554,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF060701-7CA0-45C0-BD16-F41A6A5DB4E0}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:D4"/>
@@ -819,35 +562,35 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C1" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="D1" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C3" t="b">
         <v>0</v>
@@ -855,10 +598,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C4" t="b">
         <v>0</v>

</xml_diff>